<commit_message>
Enhance estimate functions to auto-calculate labor cost based on roof area and refine labor component identification
</commit_message>
<xml_diff>
--- a/Component Metrics AI Replacement Calculator Per Roof Material Type.xlsx
+++ b/Component Metrics AI Replacement Calculator Per Roof Material Type.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hncapitalpartners-my.sharepoint.com/personal/nnambiar_hncapitalpartners_com/Documents/Documents/Personal/Fair-Price-Roof.io/Price Estimate Modelling/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Aditya.Abhiwan\FPR\data by client\AI Estimator for Retail Roof Replacements (1)\ai-estimator-losgic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE870275-142A-48F7-8DF8-85842EA274E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A5A1192-1B06-4234-B259-1A76D878ACDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{17A136AC-3DA5-4F6E-8DA3-F463D02431C9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{17A136AC-3DA5-4F6E-8DA3-F463D02431C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Shingle (Class 3)" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="168">
   <si>
     <t>Material</t>
   </si>
@@ -325,18 +325,9 @@
     <t xml:space="preserve">Labor </t>
   </si>
   <si>
-    <t>Price Per Unit</t>
-  </si>
-  <si>
     <t>Box</t>
   </si>
   <si>
-    <t>$55-$120</t>
-  </si>
-  <si>
-    <t>$89-$120</t>
-  </si>
-  <si>
     <t xml:space="preserve">Bundle  </t>
   </si>
   <si>
@@ -346,24 +337,12 @@
     <t>Eave Trim</t>
   </si>
   <si>
-    <t>$19.50-$446</t>
-  </si>
-  <si>
-    <t>$20-$44</t>
-  </si>
-  <si>
-    <t>$8-$16</t>
-  </si>
-  <si>
     <t>Z Bar</t>
   </si>
   <si>
     <t>Valley Tray</t>
   </si>
   <si>
-    <t>$17,98-$23.98</t>
-  </si>
-  <si>
     <t xml:space="preserve">Field tiles are the main tiles installed across the flat areas of roof. Class 4 rating means these tiles have been tested to withstand larger hail impacts than standard concrete or clay tiles. </t>
   </si>
   <si>
@@ -551,6 +530,21 @@
   </si>
   <si>
     <t>Plastic cement is a thick, asphalt‑based adhesive used in roofing to seal joints, flashings, and small repairs. It stays pliable, creating a watertight bond that resists cracking and weathering, making it ideal for patching leaks or securing materials in place.</t>
+  </si>
+  <si>
+    <t>Price for Crew to install shingles</t>
+  </si>
+  <si>
+    <t>Price for crew to install shingles</t>
+  </si>
+  <si>
+    <t>Price for crew to install materials</t>
+  </si>
+  <si>
+    <t>Price Per Unit (Lower)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -558,8 +552,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -609,12 +603,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -954,16 +948,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32E66F49-C25A-4113-A217-B17FA39259A7}">
-  <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.86328125" customWidth="1"/>
-    <col min="2" max="2" width="35.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.796875" customWidth="1"/>
-    <col min="4" max="5" width="17.86328125" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="38.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -974,13 +968,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>3</v>
+        <v>166</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>19</v>
       </c>
@@ -997,7 +991,7 @@
         <v>131.97</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -1014,7 +1008,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1031,7 +1025,7 @@
         <v>159.80000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -1047,8 +1041,11 @@
       <c r="E5" s="3">
         <v>139.5</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="I5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -1065,7 +1062,7 @@
         <v>9.1</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -1082,7 +1079,7 @@
         <v>16.98</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>39</v>
       </c>
@@ -1099,7 +1096,7 @@
         <v>44.31</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -1116,7 +1113,7 @@
         <v>446.75</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -1133,7 +1130,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
@@ -1150,7 +1147,7 @@
         <v>65.25</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
@@ -1167,7 +1164,7 @@
         <v>122.9</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
@@ -1184,7 +1181,7 @@
         <v>17.3</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
@@ -1201,7 +1198,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
@@ -1218,7 +1215,7 @@
         <v>8.07</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>17</v>
       </c>
@@ -1235,7 +1232,7 @@
         <v>8.9600000000000009</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>18</v>
       </c>
@@ -1250,6 +1247,23 @@
       </c>
       <c r="E17" s="3">
         <v>23.98</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C18" t="s">
+        <v>145</v>
+      </c>
+      <c r="D18" s="2">
+        <v>75</v>
+      </c>
+      <c r="E18" s="2">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1259,16 +1273,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{240CDC72-E23E-45D4-BA55-DB36E68A7E2B}">
-  <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.86328125" customWidth="1"/>
-    <col min="2" max="2" width="35.6640625" customWidth="1"/>
-    <col min="3" max="3" width="17.86328125" customWidth="1"/>
-    <col min="4" max="5" width="17.796875" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="35.7109375" customWidth="1"/>
+    <col min="3" max="5" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1285,7 +1298,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>19</v>
       </c>
@@ -1302,7 +1315,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" ht="120" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -1319,7 +1332,7 @@
         <v>132.55000000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1336,7 +1349,7 @@
         <v>159.80000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -1353,7 +1366,7 @@
         <v>139.5</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -1370,7 +1383,7 @@
         <v>9.1</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -1387,7 +1400,7 @@
         <v>16.98</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>39</v>
       </c>
@@ -1404,7 +1417,7 @@
         <v>44.31</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -1421,7 +1434,7 @@
         <v>446.75</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -1438,7 +1451,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
@@ -1455,7 +1468,7 @@
         <v>65.25</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
@@ -1472,7 +1485,7 @@
         <v>122.9</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
@@ -1489,7 +1502,7 @@
         <v>17.3</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
@@ -1506,7 +1519,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
@@ -1523,7 +1536,7 @@
         <v>8.07</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>17</v>
       </c>
@@ -1540,7 +1553,7 @@
         <v>8.9600000000000009</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>18</v>
       </c>
@@ -1555,6 +1568,23 @@
       </c>
       <c r="E17" s="5">
         <v>23.98</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D18" s="2">
+        <v>75</v>
+      </c>
+      <c r="E18" s="2">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1564,16 +1594,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B860DE0A-EE6D-493F-8697-34D873F5C8FF}">
-  <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.796875" customWidth="1"/>
-    <col min="2" max="2" width="35.46484375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="35.42578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="17.796875" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1584,15 +1615,18 @@
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="71.25" x14ac:dyDescent="0.45">
+        <v>166</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="C2" t="s">
         <v>24</v>
@@ -1600,22 +1634,28 @@
       <c r="D2" s="3">
         <v>7.41</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="E2" s="3">
+        <v>7.41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="120" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D3" s="3">
         <v>230.05</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="E3" s="3">
+        <v>230.05</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1625,11 +1665,14 @@
       <c r="C4" t="s">
         <v>61</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="D4" s="2">
+        <v>89</v>
+      </c>
+      <c r="E4" s="2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -1639,16 +1682,19 @@
       <c r="C5" t="s">
         <v>62</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="2">
+        <v>55</v>
+      </c>
+      <c r="E5" s="2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
-      <c r="A6" s="1" t="s">
-        <v>99</v>
-      </c>
       <c r="B6" s="1" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="C6" t="s">
         <v>24</v>
@@ -1656,13 +1702,16 @@
       <c r="D6" s="2">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="E6" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="C7" t="s">
         <v>24</v>
@@ -1670,8 +1719,11 @@
       <c r="D7" s="3">
         <v>7.73</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="E7" s="3">
+        <v>7.73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
@@ -1681,11 +1733,14 @@
       <c r="C8" t="s">
         <v>24</v>
       </c>
-      <c r="D8" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="57" x14ac:dyDescent="0.45">
+      <c r="D8" s="2">
+        <v>8</v>
+      </c>
+      <c r="E8" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>39</v>
       </c>
@@ -1695,11 +1750,14 @@
       <c r="C9" t="s">
         <v>24</v>
       </c>
-      <c r="D9" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="71.25" x14ac:dyDescent="0.45">
+      <c r="D9" s="2">
+        <v>20</v>
+      </c>
+      <c r="E9" s="2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1709,25 +1767,31 @@
       <c r="C10" t="s">
         <v>24</v>
       </c>
-      <c r="D10" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="99.75" x14ac:dyDescent="0.45">
+      <c r="D10" s="3">
+        <v>19.5</v>
+      </c>
+      <c r="E10" s="2">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="120" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>54</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C11" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D11" s="3">
         <v>119.28</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="71.25" x14ac:dyDescent="0.45">
+      <c r="E11" s="3">
+        <v>119.28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>12</v>
       </c>
@@ -1740,13 +1804,16 @@
       <c r="D12" s="3">
         <v>65.25</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="E12" s="3">
+        <v>65.25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="C13" t="s">
         <v>24</v>
@@ -1754,13 +1821,16 @@
       <c r="D13" s="3">
         <v>7.73</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="71.25" x14ac:dyDescent="0.45">
+      <c r="E13" s="3">
+        <v>7.73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C14" t="s">
         <v>24</v>
@@ -1768,8 +1838,11 @@
       <c r="D14" s="3">
         <v>8.64</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="E14" s="3">
+        <v>8.64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -1782,13 +1855,16 @@
       <c r="D15" s="2">
         <v>17</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="57" x14ac:dyDescent="0.45">
+      <c r="E15" s="2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="C16" t="s">
         <v>24</v>
@@ -1796,8 +1872,11 @@
       <c r="D16" s="3">
         <v>3.1</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="57" x14ac:dyDescent="0.45">
+      <c r="E16" s="3">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
@@ -1810,13 +1889,16 @@
       <c r="D17" s="3">
         <v>8.8699999999999992</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="57" x14ac:dyDescent="0.45">
+      <c r="E17" s="3">
+        <v>8.8699999999999992</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="C18" t="s">
         <v>23</v>
@@ -1824,13 +1906,16 @@
       <c r="D18" s="3">
         <v>1.55</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="E18" s="3">
+        <v>1.55</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="C19" t="s">
         <v>27</v>
@@ -1838,27 +1923,33 @@
       <c r="D19" s="3">
         <v>304.10000000000002</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="E19" s="3">
+        <v>304.10000000000002</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C20" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D20" s="3">
         <v>191.3</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="57" x14ac:dyDescent="0.45">
+      <c r="E20" s="3">
+        <v>191.3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="C21" t="s">
         <v>24</v>
@@ -1866,8 +1957,11 @@
       <c r="D21" s="3">
         <v>4.55</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="57" x14ac:dyDescent="0.45">
+      <c r="E21" s="3">
+        <v>4.55</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>60</v>
       </c>
@@ -1877,8 +1971,28 @@
       <c r="C22" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>106</v>
+      <c r="D22" s="2">
+        <v>17.98</v>
+      </c>
+      <c r="E22" s="3">
+        <v>23.98</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C23" t="s">
+        <v>149</v>
+      </c>
+      <c r="D23" s="2">
+        <v>200</v>
+      </c>
+      <c r="E23" s="2">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -1888,17 +2002,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4344B64-734B-483E-B5CE-15D09E3A0208}">
-  <dimension ref="A1:E18"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.796875" customWidth="1"/>
-    <col min="2" max="2" width="26.6640625" customWidth="1"/>
-    <col min="3" max="3" width="17.796875" customWidth="1"/>
-    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1915,15 +2029,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B2" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="C2" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="D2" s="3">
         <v>41.05</v>
@@ -1932,15 +2046,15 @@
         <v>41.05</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="C3" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="D3" s="3">
         <v>69.78</v>
@@ -1949,7 +2063,7 @@
         <v>69.78</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1966,7 +2080,7 @@
         <v>159.80000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" ht="135" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -1983,7 +2097,7 @@
         <v>139.5</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="114" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -2000,7 +2114,7 @@
         <v>9.1</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" ht="135" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -2017,7 +2131,7 @@
         <v>16.98</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>39</v>
       </c>
@@ -2034,7 +2148,7 @@
         <v>44.31</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:5" ht="120" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -2051,21 +2165,24 @@
         <v>446.75</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="114" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" ht="135" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>64</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="C10" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D10" s="3">
         <v>51.3</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="99.75" x14ac:dyDescent="0.45">
+      <c r="E10" s="3">
+        <v>51.3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="135" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
@@ -2082,7 +2199,7 @@
         <v>65.25</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
@@ -2099,7 +2216,7 @@
         <v>122.9</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="114" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:5" ht="135" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
@@ -2116,7 +2233,7 @@
         <v>17.3</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
@@ -2133,7 +2250,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
@@ -2150,7 +2267,7 @@
         <v>8.07</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>17</v>
       </c>
@@ -2167,15 +2284,15 @@
         <v>8.9600000000000009</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="C17" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="D17" s="3">
         <v>58.24</v>
@@ -2184,7 +2301,7 @@
         <v>58.24</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>60</v>
       </c>
@@ -2199,6 +2316,23 @@
       </c>
       <c r="E18" s="5">
         <v>23.98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D19" s="2">
+        <v>200</v>
+      </c>
+      <c r="E19" s="2">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -2209,16 +2343,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAEFCB5B-60D6-4E73-9873-3C11287D2130}">
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.796875" customWidth="1"/>
-    <col min="2" max="2" width="26.6640625" customWidth="1"/>
-    <col min="3" max="3" width="17.796875" customWidth="1"/>
-    <col min="4" max="4" width="17.86328125" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="88" customWidth="1"/>
+    <col min="3" max="4" width="17.85546875" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -2235,26 +2368,29 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="285" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="C2" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="D2" s="3">
         <v>715.79</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="242.25" x14ac:dyDescent="0.45">
+      <c r="E2" s="3">
+        <v>715.79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="C3" t="s">
         <v>62</v>
@@ -2262,27 +2398,33 @@
       <c r="D3" s="3">
         <v>389.25</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="228" x14ac:dyDescent="0.45">
+      <c r="E3" s="3">
+        <v>389.25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="C4" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="D4" s="3">
         <v>118.32</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="114" x14ac:dyDescent="0.45">
+      <c r="E4" s="3">
+        <v>118.32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>69</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C5" t="s">
         <v>29</v>
@@ -2290,27 +2432,33 @@
       <c r="D5" s="3">
         <v>30.39</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="156.75" x14ac:dyDescent="0.45">
+      <c r="E5" s="3">
+        <v>30.39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>70</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C6" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="D6" s="2">
         <v>614</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="156.75" x14ac:dyDescent="0.45">
+      <c r="E6" s="2">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="C7" t="s">
         <v>24</v>
@@ -2318,13 +2466,16 @@
       <c r="D7" s="3">
         <v>43.03</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="156.75" x14ac:dyDescent="0.45">
+      <c r="E7" s="3">
+        <v>43.03</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="C8" t="s">
         <v>24</v>
@@ -2332,55 +2483,67 @@
       <c r="D8" s="3">
         <v>41.43</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="142.5" x14ac:dyDescent="0.45">
+      <c r="E8" s="3">
+        <v>41.43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>72</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="C9" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="D9" s="3">
         <v>12.29</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="128.25" x14ac:dyDescent="0.45">
+      <c r="E9" s="3">
+        <v>12.29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>73</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C10" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="D10" s="3">
         <v>161.91999999999999</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="156.75" x14ac:dyDescent="0.45">
+      <c r="E10" s="3">
+        <v>161.91999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="C11" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="D11" s="3">
         <v>509.94</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="142.5" x14ac:dyDescent="0.45">
+      <c r="E11" s="3">
+        <v>509.94</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>75</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="C12" t="s">
         <v>24</v>
@@ -2388,41 +2551,50 @@
       <c r="D12" s="3">
         <v>12.5</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="128.25" x14ac:dyDescent="0.45">
+      <c r="E12" s="3">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>76</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="C13" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="D13" s="3">
         <v>51.22</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" ht="142.5" x14ac:dyDescent="0.45">
+      <c r="E13" s="3">
+        <v>51.22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>77</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="C14" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="D14" s="3">
         <v>21.59</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" ht="156.75" x14ac:dyDescent="0.45">
+      <c r="E14" s="3">
+        <v>21.59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>78</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="C15" t="s">
         <v>24</v>
@@ -2430,27 +2602,33 @@
       <c r="D15" s="3">
         <v>8.69</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" ht="128.25" x14ac:dyDescent="0.45">
+      <c r="E15" s="3">
+        <v>8.69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="C16" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="D16" s="3">
         <v>17.29</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="142.5" x14ac:dyDescent="0.45">
+      <c r="E16" s="3">
+        <v>17.29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>79</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="C17" t="s">
         <v>24</v>
@@ -2458,30 +2636,36 @@
       <c r="D17" s="3">
         <v>120.14</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" ht="156.75" x14ac:dyDescent="0.45">
+      <c r="E17" s="3">
+        <v>120.14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C18" t="s">
         <v>144</v>
-      </c>
-      <c r="C18" t="s">
-        <v>151</v>
       </c>
       <c r="D18" s="3">
         <v>676.75</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" ht="142.5" x14ac:dyDescent="0.45">
+      <c r="E18" s="3">
+        <v>676.75</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>81</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C19" t="s">
         <v>145</v>
-      </c>
-      <c r="C19" t="s">
-        <v>152</v>
       </c>
       <c r="D19" s="2">
         <v>150</v>
@@ -2498,16 +2682,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C77F6F8-A634-4692-9CC0-75300D99772E}">
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.796875" customWidth="1"/>
-    <col min="2" max="2" width="26.796875" customWidth="1"/>
-    <col min="3" max="3" width="17.6640625" customWidth="1"/>
-    <col min="4" max="4" width="17.796875" customWidth="1"/>
-    <col min="5" max="5" width="17.86328125" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" customWidth="1"/>
+    <col min="4" max="5" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -2524,15 +2707,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="114" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:5" ht="135" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>82</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="C2" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D2" s="2">
         <v>100</v>
@@ -2541,29 +2724,32 @@
         <v>125</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" ht="165" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>83</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="C3" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="D3" s="2">
         <v>131</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="128.25" x14ac:dyDescent="0.45">
+      <c r="E3" s="2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>84</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="C4" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="D4" s="2">
         <v>60</v>
@@ -2572,71 +2758,80 @@
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="114" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>85</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C5" t="s">
         <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="E5" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="156.75" x14ac:dyDescent="0.45">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="180" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>70</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C6" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="D6" s="3">
         <v>380.71</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="128.25" x14ac:dyDescent="0.45">
+      <c r="E6" s="3">
+        <v>380.71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>86</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="C7" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D7" s="2">
         <v>120</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E7" s="2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>87</v>
       </c>
       <c r="B8" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="C8" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="D8" s="3">
         <v>14.73</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="142.5" x14ac:dyDescent="0.45">
+      <c r="E8" s="3">
+        <v>14.73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="180" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>88</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="C9" t="s">
         <v>24</v>
@@ -2648,40 +2843,46 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" ht="180" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="C10" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="D10" s="3">
         <v>63.53</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="142.5" x14ac:dyDescent="0.45">
+      <c r="E10" s="3">
+        <v>63.53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="195" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>72</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="C11" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="D11" s="3">
         <v>10.45</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="114" x14ac:dyDescent="0.45">
+      <c r="E11" s="3">
+        <v>10.45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="C12" t="s">
         <v>24</v>
@@ -2689,13 +2890,16 @@
       <c r="D12" s="3">
         <v>8.15</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="142.5" x14ac:dyDescent="0.45">
+      <c r="E12" s="3">
+        <v>8.15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="165" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>79</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="C13" t="s">
         <v>24</v>
@@ -2703,16 +2907,19 @@
       <c r="D13" s="3">
         <v>120.15</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" ht="114" x14ac:dyDescent="0.45">
+      <c r="E13" s="3">
+        <v>120.15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>91</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="C14" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="D14" s="2">
         <v>59</v>
@@ -2721,15 +2928,15 @@
         <v>82</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="114" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" ht="150" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="C15" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="D15" s="2">
         <v>60</v>
@@ -2738,15 +2945,15 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="142.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:5" ht="165" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>93</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="C16" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="D16" s="2">
         <v>150</v>

</xml_diff>

<commit_message>
Refactor tax handling in pricing calculations to use tax rate instead of fixed taxes, update related variables and tests accordingly
</commit_message>
<xml_diff>
--- a/Component Metrics AI Replacement Calculator Per Roof Material Type.xlsx
+++ b/Component Metrics AI Replacement Calculator Per Roof Material Type.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Aditya.Abhiwan\FPR\data by client\AI Estimator for Retail Roof Replacements (1)\ai-estimator-losgic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A5A1192-1B06-4234-B259-1A76D878ACDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE5B60B6-24F1-4063-8518-6E773807548E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{17A136AC-3DA5-4F6E-8DA3-F463D02431C9}"/>
+    <workbookView xWindow="3090" yWindow="3180" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{17A136AC-3DA5-4F6E-8DA3-F463D02431C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Shingle (Class 3)" sheetId="1" r:id="rId1"/>
@@ -985,7 +985,7 @@
         <v>30</v>
       </c>
       <c r="D2" s="2">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="E2" s="3">
         <v>131.97</v>
@@ -1002,7 +1002,7 @@
         <v>31</v>
       </c>
       <c r="D3" s="2">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E3" s="3">
         <v>116</v>
@@ -1312,7 +1312,7 @@
         <v>125</v>
       </c>
       <c r="E2" s="5">
-        <v>173</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="120" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add new roof material calculators and JSON data files
- Introduced JSON files for Synthetic Tile (Brava) and TPO roof materials, detailing components, descriptions, units of measurement, and pricing.
- Created an index file to reference all roof material types and their respective JSON files.
- Implemented a new module structure for roof type calculators, including common utilities and specific calculators for each roof type.
- Added quantity calculation functions for various roofing components, ensuring accurate estimates based on roof area and complexity.
- Enhanced the registry to link components with their respective calculators for streamlined access.
</commit_message>
<xml_diff>
--- a/Component Metrics AI Replacement Calculator Per Roof Material Type.xlsx
+++ b/Component Metrics AI Replacement Calculator Per Roof Material Type.xlsx
@@ -5,20 +5,21 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Aditya.Abhiwan\FPR\data by client\AI Estimator for Retail Roof Replacements (1)\ai-estimator-losgic\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE5B60B6-24F1-4063-8518-6E773807548E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3432776A-FE42-40DD-A87A-1DD5A66EAFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3090" yWindow="3180" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{17A136AC-3DA5-4F6E-8DA3-F463D02431C9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{17A136AC-3DA5-4F6E-8DA3-F463D02431C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Shingle (Class 3)" sheetId="1" r:id="rId1"/>
     <sheet name="Shingles (Class 4)" sheetId="2" r:id="rId2"/>
     <sheet name="Stone Coated Steel" sheetId="3" r:id="rId3"/>
-    <sheet name="Synthetic Tile (Brava)" sheetId="4" r:id="rId4"/>
-    <sheet name="TPO" sheetId="5" r:id="rId5"/>
-    <sheet name="Modified" sheetId="6" r:id="rId6"/>
+    <sheet name="Standing Seam" sheetId="7" r:id="rId4"/>
+    <sheet name="Synthetic Tile (Brava)" sheetId="4" r:id="rId5"/>
+    <sheet name="TPO" sheetId="5" r:id="rId6"/>
+    <sheet name="Modified" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="171">
   <si>
     <t>Material</t>
   </si>
@@ -379,12 +380,6 @@
     <t>Granules are installed on top of caulking to ensure a similar texture to the stone-coated steel panels at all seams. It also protects the caulking from UV rays.</t>
   </si>
   <si>
-    <t>Bundle (12 Pieces)</t>
-  </si>
-  <si>
-    <t>Bundle (10 Pieces)</t>
-  </si>
-  <si>
     <t>Roll (1 square)</t>
   </si>
   <si>
@@ -460,9 +455,6 @@
     <t>Labor refers to the skilled work performed by roofing crews during installation or repair. It includes tasks such as preparing the roof deck, installing insulation, fastening membranes, and sealing details. Quality labor ensures the roofing system is installed correctly, watertight, and built to last.</t>
   </si>
   <si>
-    <t>Roll (100 Squares)</t>
-  </si>
-  <si>
     <t>5 Gal</t>
   </si>
   <si>
@@ -541,10 +533,28 @@
     <t>Price for crew to install materials</t>
   </si>
   <si>
-    <t>Price Per Unit (Lower)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
+    <t>For standing seam, we pay one price for material and labor</t>
+  </si>
+  <si>
+    <t>Price per Square</t>
+  </si>
+  <si>
+    <t>Tear Off</t>
+  </si>
+  <si>
+    <t>To tear off existing shingle roof</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decking is the solid surface, usually made of plywood or OSB, that forms the bec of the roof. It provides structural support for shingles and roofing materials. </t>
+  </si>
+  <si>
+    <t>Material and Labor</t>
+  </si>
+  <si>
+    <t>Price Per Unit(Lower)</t>
+  </si>
+  <si>
+    <t>Price Per Unit(Upper)</t>
   </si>
 </sst>
 </file>
@@ -598,7 +608,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -614,6 +624,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -948,16 +959,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32E66F49-C25A-4113-A217-B17FA39259A7}">
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" customWidth="1"/>
-    <col min="2" max="2" width="38.5703125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="35.7109375" style="1" customWidth="1"/>
+    <col min="3" max="5" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -968,13 +978,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>166</v>
+        <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>19</v>
       </c>
@@ -985,13 +995,13 @@
         <v>30</v>
       </c>
       <c r="D2" s="2">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="E2" s="3">
         <v>131.97</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -1002,13 +1012,13 @@
         <v>31</v>
       </c>
       <c r="D3" s="2">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E3" s="3">
         <v>116</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1025,7 +1035,7 @@
         <v>159.80000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -1041,11 +1051,8 @@
       <c r="E5" s="3">
         <v>139.5</v>
       </c>
-      <c r="I5" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -1062,7 +1069,7 @@
         <v>9.1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -1079,7 +1086,7 @@
         <v>16.98</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>39</v>
       </c>
@@ -1096,7 +1103,7 @@
         <v>44.31</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -1113,7 +1120,7 @@
         <v>446.75</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -1130,7 +1137,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="105" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
@@ -1147,7 +1154,7 @@
         <v>65.25</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>13</v>
       </c>
@@ -1164,7 +1171,7 @@
         <v>122.9</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
@@ -1181,7 +1188,7 @@
         <v>17.3</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
@@ -1198,7 +1205,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
@@ -1215,7 +1222,7 @@
         <v>8.07</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>17</v>
       </c>
@@ -1243,10 +1250,10 @@
         <v>29</v>
       </c>
       <c r="D17" s="3">
-        <v>17.98</v>
+        <v>18</v>
       </c>
       <c r="E17" s="3">
-        <v>23.98</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1254,16 +1261,16 @@
         <v>93</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="C18" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D18" s="2">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E18" s="2">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1312,7 +1319,7 @@
         <v>125</v>
       </c>
       <c r="E2" s="5">
-        <v>165</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="120" x14ac:dyDescent="0.25">
@@ -1564,10 +1571,10 @@
         <v>29</v>
       </c>
       <c r="D17" s="5">
-        <v>17.98</v>
+        <v>18</v>
       </c>
       <c r="E17" s="5">
-        <v>23.98</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1575,16 +1582,16 @@
         <v>81</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D18" s="2">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E18" s="2">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1600,11 +1607,11 @@
     <col min="1" max="1" width="17.85546875" customWidth="1"/>
     <col min="2" max="2" width="35.42578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" customWidth="1"/>
+    <col min="4" max="4" width="24.85546875" customWidth="1"/>
+    <col min="5" max="5" width="27.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1615,10 +1622,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>4</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="75" x14ac:dyDescent="0.25">
@@ -1629,13 +1636,13 @@
         <v>100</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>146</v>
       </c>
       <c r="D2" s="3">
-        <v>7.41</v>
-      </c>
-      <c r="E2" s="3">
-        <v>7.41</v>
+        <v>180</v>
+      </c>
+      <c r="E2" s="2">
+        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="120" x14ac:dyDescent="0.25">
@@ -1966,16 +1973,16 @@
         <v>60</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>49</v>
+        <v>167</v>
       </c>
       <c r="C22" t="s">
         <v>24</v>
       </c>
       <c r="D22" s="2">
-        <v>17.98</v>
+        <v>20</v>
       </c>
       <c r="E22" s="3">
-        <v>23.98</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -1983,16 +1990,102 @@
         <v>81</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C23" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D23" s="2">
         <v>200</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="3">
         <v>250</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="70" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F554FB00-CA27-4018-A37D-529C6B635178}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" customWidth="1"/>
+    <col min="4" max="4" width="22.140625" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D2" s="2">
+        <v>680</v>
+      </c>
+      <c r="E2" s="2">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C3" t="s">
+        <v>164</v>
+      </c>
+      <c r="D3" s="2">
+        <v>30</v>
+      </c>
+      <c r="E3" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="150" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="2">
+        <v>18</v>
+      </c>
+      <c r="E4" s="2">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -2000,7 +2093,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4344B64-734B-483E-B5CE-15D09E3A0208}">
   <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2034,16 +2127,18 @@
         <v>52</v>
       </c>
       <c r="B2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C2" t="s">
-        <v>112</v>
+        <v>146</v>
       </c>
       <c r="D2" s="3">
-        <v>41.05</v>
+        <f>41.05*7</f>
+        <v>287.34999999999997</v>
       </c>
       <c r="E2" s="3">
-        <v>41.05</v>
+        <f>41.05*8</f>
+        <v>328.4</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -2051,16 +2146,18 @@
         <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>146</v>
       </c>
       <c r="D3" s="3">
-        <v>69.78</v>
+        <f>69.78*8</f>
+        <v>558.24</v>
       </c>
       <c r="E3" s="3">
-        <v>69.78</v>
+        <f>69.78*9</f>
+        <v>628.02</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="75" x14ac:dyDescent="0.25">
@@ -2170,10 +2267,10 @@
         <v>64</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D10" s="3">
         <v>51.3</v>
@@ -2289,10 +2386,10 @@
         <v>65</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C17" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D17" s="3">
         <v>58.24</v>
@@ -2312,10 +2409,10 @@
         <v>29</v>
       </c>
       <c r="D18" s="5">
-        <v>17.98</v>
+        <v>18</v>
       </c>
       <c r="E18" s="5">
-        <v>23.98</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" x14ac:dyDescent="0.25">
@@ -2323,355 +2420,16 @@
         <v>81</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D19" s="2">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="E19" s="2">
-        <v>250</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAEFCB5B-60D6-4E73-9873-3C11287D2130}">
-  <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="17.85546875" customWidth="1"/>
-    <col min="2" max="2" width="88" customWidth="1"/>
-    <col min="3" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="105" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="C2" t="s">
-        <v>139</v>
-      </c>
-      <c r="D2" s="3">
-        <v>715.79</v>
-      </c>
-      <c r="E2" s="3">
-        <v>715.79</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="90" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D3" s="3">
-        <v>389.25</v>
-      </c>
-      <c r="E3" s="3">
-        <v>389.25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="90" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="C4" t="s">
-        <v>140</v>
-      </c>
-      <c r="D4" s="3">
-        <v>118.32</v>
-      </c>
-      <c r="E4" s="3">
-        <v>118.32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="C5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="3">
-        <v>30.39</v>
-      </c>
-      <c r="E5" s="3">
-        <v>30.39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C6" t="s">
-        <v>141</v>
-      </c>
-      <c r="D6" s="2">
-        <v>614</v>
-      </c>
-      <c r="E6" s="2">
-        <v>614</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="C7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="3">
-        <v>43.03</v>
-      </c>
-      <c r="E7" s="3">
-        <v>43.03</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="3">
-        <v>41.43</v>
-      </c>
-      <c r="E8" s="3">
-        <v>41.43</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="C9" t="s">
-        <v>143</v>
-      </c>
-      <c r="D9" s="3">
-        <v>12.29</v>
-      </c>
-      <c r="E9" s="3">
-        <v>12.29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="C10" t="s">
-        <v>140</v>
-      </c>
-      <c r="D10" s="3">
-        <v>161.91999999999999</v>
-      </c>
-      <c r="E10" s="3">
-        <v>161.91999999999999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="C11" t="s">
-        <v>141</v>
-      </c>
-      <c r="D11" s="3">
-        <v>509.94</v>
-      </c>
-      <c r="E11" s="3">
-        <v>509.94</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="C12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="3">
-        <v>12.5</v>
-      </c>
-      <c r="E12" s="3">
-        <v>12.5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="C13" t="s">
-        <v>142</v>
-      </c>
-      <c r="D13" s="3">
-        <v>51.22</v>
-      </c>
-      <c r="E13" s="3">
-        <v>51.22</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C14" t="s">
-        <v>146</v>
-      </c>
-      <c r="D14" s="3">
-        <v>21.59</v>
-      </c>
-      <c r="E14" s="3">
-        <v>21.59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="C15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="3">
-        <v>8.69</v>
-      </c>
-      <c r="E15" s="3">
-        <v>8.69</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="45" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="C16" t="s">
-        <v>143</v>
-      </c>
-      <c r="D16" s="3">
-        <v>17.29</v>
-      </c>
-      <c r="E16" s="3">
-        <v>17.29</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="C17" t="s">
-        <v>24</v>
-      </c>
-      <c r="D17" s="3">
-        <v>120.14</v>
-      </c>
-      <c r="E17" s="3">
-        <v>120.14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="C18" t="s">
-        <v>144</v>
-      </c>
-      <c r="D18" s="3">
-        <v>676.75</v>
-      </c>
-      <c r="E18" s="3">
-        <v>676.75</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="60" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="C19" t="s">
-        <v>145</v>
-      </c>
-      <c r="D19" s="2">
-        <v>150</v>
-      </c>
-      <c r="E19" s="2">
-        <v>200</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -2680,6 +2438,346 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAEFCB5B-60D6-4E73-9873-3C11287D2130}">
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" customWidth="1"/>
+    <col min="3" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="360" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" s="3">
+        <v>715.79</v>
+      </c>
+      <c r="E2" s="3">
+        <v>715.79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="300" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D3" s="3">
+        <v>389.25</v>
+      </c>
+      <c r="E3" s="3">
+        <v>389.25</v>
+      </c>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="1:6" ht="270" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D4" s="3">
+        <v>118.32</v>
+      </c>
+      <c r="E4" s="3">
+        <v>118.32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="150" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="3">
+        <v>30.39</v>
+      </c>
+      <c r="E5" s="3">
+        <v>30.39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="180" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D6" s="2">
+        <v>614</v>
+      </c>
+      <c r="E6" s="2">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="210" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="3">
+        <v>43.03</v>
+      </c>
+      <c r="E7" s="3">
+        <v>43.03</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="195" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="3">
+        <v>41.43</v>
+      </c>
+      <c r="E8" s="3">
+        <v>41.43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="195" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" t="s">
+        <v>140</v>
+      </c>
+      <c r="D9" s="3">
+        <v>12.29</v>
+      </c>
+      <c r="E9" s="3">
+        <v>12.29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="165" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D10" s="3">
+        <v>161.91999999999999</v>
+      </c>
+      <c r="E10" s="3">
+        <v>161.91999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="195" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C11" t="s">
+        <v>138</v>
+      </c>
+      <c r="D11" s="3">
+        <v>509.94</v>
+      </c>
+      <c r="E11" s="3">
+        <v>509.94</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="180" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="3">
+        <v>12.5</v>
+      </c>
+      <c r="E12" s="3">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="165" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C13" t="s">
+        <v>139</v>
+      </c>
+      <c r="D13" s="3">
+        <v>51.22</v>
+      </c>
+      <c r="E13" s="3">
+        <v>51.22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="165" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C14" t="s">
+        <v>143</v>
+      </c>
+      <c r="D14" s="3">
+        <v>21.59</v>
+      </c>
+      <c r="E14" s="3">
+        <v>21.59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="180" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C15" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="3">
+        <v>8.69</v>
+      </c>
+      <c r="E15" s="3">
+        <v>8.69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="165" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C16" t="s">
+        <v>140</v>
+      </c>
+      <c r="D16" s="3">
+        <v>17.29</v>
+      </c>
+      <c r="E16" s="3">
+        <v>17.29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="180" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C17" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" s="3">
+        <v>120.14</v>
+      </c>
+      <c r="E17" s="3">
+        <v>120.14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="180" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C18" t="s">
+        <v>141</v>
+      </c>
+      <c r="D18" s="3">
+        <v>676.75</v>
+      </c>
+      <c r="E18" s="3">
+        <v>676.75</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="165" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C19" t="s">
+        <v>142</v>
+      </c>
+      <c r="D19" s="2">
+        <v>150</v>
+      </c>
+      <c r="E19" s="2">
+        <v>200</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C77F6F8-A634-4692-9CC0-75300D99772E}">
   <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2712,10 +2810,10 @@
         <v>82</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D2" s="2">
         <v>100</v>
@@ -2729,10 +2827,10 @@
         <v>83</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C3" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D3" s="2">
         <v>131</v>
@@ -2746,10 +2844,10 @@
         <v>84</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C4" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D4" s="2">
         <v>60</v>
@@ -2763,16 +2861,16 @@
         <v>85</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C5" t="s">
         <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="180" x14ac:dyDescent="0.25">
@@ -2780,10 +2878,10 @@
         <v>70</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C6" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D6" s="3">
         <v>380.71</v>
@@ -2797,10 +2895,10 @@
         <v>86</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D7" s="2">
         <v>120</v>
@@ -2814,10 +2912,10 @@
         <v>87</v>
       </c>
       <c r="B8" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C8" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D8" s="3">
         <v>14.73</v>
@@ -2831,7 +2929,7 @@
         <v>88</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C9" t="s">
         <v>24</v>
@@ -2848,10 +2946,10 @@
         <v>89</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C10" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D10" s="3">
         <v>63.53</v>
@@ -2865,10 +2963,10 @@
         <v>72</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C11" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D11" s="3">
         <v>10.45</v>
@@ -2882,7 +2980,7 @@
         <v>90</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C12" t="s">
         <v>24</v>
@@ -2899,7 +2997,7 @@
         <v>79</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C13" t="s">
         <v>24</v>
@@ -2916,10 +3014,10 @@
         <v>91</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C14" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D14" s="2">
         <v>59</v>
@@ -2933,10 +3031,10 @@
         <v>92</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C15" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D15" s="2">
         <v>60</v>
@@ -2950,10 +3048,10 @@
         <v>93</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C16" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D16" s="2">
         <v>150</v>

</xml_diff>

<commit_message>
Add standing seam roof type calculations and related tests
</commit_message>
<xml_diff>
--- a/Component Metrics AI Replacement Calculator Per Roof Material Type.xlsx
+++ b/Component Metrics AI Replacement Calculator Per Roof Material Type.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Aditya.Abhiwan\FPR\data by client\AI Estimator for Retail Roof Replacements (1)\ai-estimator-losgic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3432776A-FE42-40DD-A87A-1DD5A66EAFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FD8EF9A-11EA-4D02-9C4F-3F6BA848E076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{17A136AC-3DA5-4F6E-8DA3-F463D02431C9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{17A136AC-3DA5-4F6E-8DA3-F463D02431C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Shingle (Class 3)" sheetId="1" r:id="rId1"/>
@@ -624,7 +624,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2017,7 +2017,7 @@
     <col min="2" max="2" width="17.85546875" customWidth="1"/>
     <col min="3" max="3" width="26.5703125" customWidth="1"/>
     <col min="4" max="4" width="22.140625" customWidth="1"/>
-    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="5" max="5" width="21" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2034,7 +2034,7 @@
         <v>169</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="60" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Refactor quantity calculations to use math.ceil for rounding and enhance price parsing for dollar amounts
</commit_message>
<xml_diff>
--- a/Component Metrics AI Replacement Calculator Per Roof Material Type.xlsx
+++ b/Component Metrics AI Replacement Calculator Per Roof Material Type.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Aditya.Abhiwan\FPR\data by client\AI Estimator for Retail Roof Replacements (1)\ai-estimator-losgic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FD8EF9A-11EA-4D02-9C4F-3F6BA848E076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{977C18FD-E6C4-47EE-B603-85989F9E8817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{17A136AC-3DA5-4F6E-8DA3-F463D02431C9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{17A136AC-3DA5-4F6E-8DA3-F463D02431C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Shingle (Class 3)" sheetId="1" r:id="rId1"/>
@@ -488,9 +488,6 @@
     <t>1" thick $17.39</t>
   </si>
   <si>
-    <t>2.2" thick $2976</t>
-  </si>
-  <si>
     <t>Bundle (96 Linear feet)</t>
   </si>
   <si>
@@ -555,6 +552,9 @@
   </si>
   <si>
     <t>Price Per Unit(Upper)</t>
+  </si>
+  <si>
+    <t>2.2" thick $29.76</t>
   </si>
 </sst>
 </file>
@@ -1261,7 +1261,7 @@
         <v>93</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C18" t="s">
         <v>142</v>
@@ -1582,7 +1582,7 @@
         <v>81</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>142</v>
@@ -1622,10 +1622,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>169</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="75" x14ac:dyDescent="0.25">
@@ -1973,7 +1973,7 @@
         <v>60</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C22" t="s">
         <v>24</v>
@@ -1990,7 +1990,7 @@
         <v>81</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C23" t="s">
         <v>146</v>
@@ -2031,21 +2031,21 @@
         <v>2</v>
       </c>
       <c r="D1" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>169</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C2" t="s">
         <v>163</v>
-      </c>
-      <c r="C2" t="s">
-        <v>164</v>
       </c>
       <c r="D2" s="2">
         <v>680</v>
@@ -2056,13 +2056,13 @@
     </row>
     <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="C3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D3" s="2">
         <v>30</v>
@@ -2076,7 +2076,7 @@
         <v>60</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C4" t="s">
         <v>24</v>
@@ -2420,7 +2420,7 @@
         <v>81</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>146</v>
@@ -2810,7 +2810,7 @@
         <v>82</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C2" t="s">
         <v>112</v>
@@ -2827,7 +2827,7 @@
         <v>83</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C3" t="s">
         <v>144</v>
@@ -2844,7 +2844,7 @@
         <v>84</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C4" t="s">
         <v>137</v>
@@ -2870,7 +2870,7 @@
         <v>147</v>
       </c>
       <c r="E5" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="180" x14ac:dyDescent="0.25">
@@ -2895,7 +2895,7 @@
         <v>86</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C7" t="s">
         <v>112</v>
@@ -2912,7 +2912,7 @@
         <v>87</v>
       </c>
       <c r="B8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C8" t="s">
         <v>140</v>
@@ -2929,7 +2929,7 @@
         <v>88</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C9" t="s">
         <v>24</v>
@@ -2946,10 +2946,10 @@
         <v>89</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D10" s="3">
         <v>63.53</v>
@@ -2980,7 +2980,7 @@
         <v>90</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C12" t="s">
         <v>24</v>
@@ -3014,7 +3014,7 @@
         <v>91</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C14" t="s">
         <v>145</v>
@@ -3031,7 +3031,7 @@
         <v>92</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C15" t="s">
         <v>137</v>

</xml_diff>